<commit_message>
Specs, audit and compliance workbooks brought up to date with the build (status 14 October 2026)
- EIR spec v4: 100 dated status notes and 19 marked corrections across sections 0-17; FLI spec v1:
  46 notes, 4 corrections; UI/report spec, the 9 Oct system audit (addendum with a 47-row table)
  and the two reviews carry a 14 October status; bootstrap README corrected
- Compliance workbooks regenerated: governance keys corrected (61 settings; unread keys tagged),
  RBM rebuilt from the Gazette's paragraphs (19 rows), CS1 7 new rows; build_audit.py now fails on
  an unknown governance key or a cited method that doesn't exist
- Specs re-rendered to .docx and .pdf (copies in OneDrive 3. Project Execution/specs; previous
  versions archived)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/compliance/Contract_Schedule1_Acceptance_Audit.xlsx
+++ b/docs/compliance/Contract_Schedule1_Acceptance_Audit.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Baselines" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Audit'!$A$4:$K$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Audit'!$A$4:$K$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Audit'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$4:$4</definedName>
   </definedNames>
@@ -604,7 +604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="C10" s="13">
-        <f>COUNTA(Audit!$A$5:$A$20)-3</f>
+        <f>COUNTA(Audit!$A$5:$A$27)-3</f>
         <v/>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Data onboarding</t>
+          <t>Data import and onboarding</t>
         </is>
       </c>
       <c r="C15" s="16">
@@ -799,7 +799,7 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Collateral management</t>
+          <t>Collateral module</t>
         </is>
       </c>
       <c r="C16" s="16">
@@ -820,7 +820,7 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>The effective interest rate and revenue recognition</t>
+          <t>EIR module and revenue recognition</t>
         </is>
       </c>
       <c r="C17" s="16">
@@ -841,7 +841,7 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>IFRS 9 model set-up</t>
+          <t>IFRS 9 model set-up: SICR and staging, PD, LGD, forward-looking information</t>
         </is>
       </c>
       <c r="C18" s="16">
@@ -862,7 +862,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>The ECL engine</t>
+          <t>ECL engine</t>
         </is>
       </c>
       <c r="C19" s="16">
@@ -904,7 +904,7 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>The audit trail</t>
+          <t>Audit trail</t>
         </is>
       </c>
       <c r="C21" s="16">
@@ -925,7 +925,7 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>The dashboard and the workspace</t>
+          <t>Dashboard and workspace</t>
         </is>
       </c>
       <c r="C22" s="16">
@@ -946,7 +946,7 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Administration</t>
+          <t>User and access management; operations</t>
         </is>
       </c>
       <c r="C23" s="16">
@@ -960,21 +960,35 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>DOCUMENTATION</t>
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>S1.10</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Internal grading</t>
+        </is>
+      </c>
+      <c r="C24" s="16">
+        <f>Audit!D15</f>
+        <v/>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 15</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>S1.11</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>User manual</t>
+          <t>EAD module</t>
         </is>
       </c>
       <c r="C25" s="16">
@@ -990,12 +1004,12 @@
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>S1.12</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>Administrator manual</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="C26" s="16">
@@ -1011,12 +1025,12 @@
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>S1.13</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>Technical manual and installation guide</t>
+          <t>The Mega Farm programme</t>
         </is>
       </c>
       <c r="C27" s="16">
@@ -1030,61 +1044,194 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>S1.14</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Annual report alignment</t>
+        </is>
+      </c>
+      <c r="C28" s="16">
+        <f>Audit!D19</f>
+        <v/>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>DELIVERABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Migration reconciliation report</t>
+        </is>
+      </c>
+      <c r="C30" s="16">
+        <f>Audit!D21</f>
+        <v/>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>User manual</t>
+        </is>
+      </c>
+      <c r="C31" s="16">
+        <f>Audit!D22</f>
+        <v/>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Administrator and Technical Manual</t>
+        </is>
+      </c>
+      <c r="C32" s="16">
+        <f>Audit!D23</f>
+        <v/>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Installation and Configuration Guide</t>
+        </is>
+      </c>
+      <c r="C33" s="16">
+        <f>Audit!D24</f>
+        <v/>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>Deployment, training and source code</t>
+        </is>
+      </c>
+      <c r="C34" s="16">
+        <f>Audit!D25</f>
+        <v/>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>ACCEPTANCE</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>The specification's acceptance tests</t>
         </is>
       </c>
-      <c r="C29" s="16">
-        <f>Audit!D20</f>
-        <v/>
-      </c>
-      <c r="D29" s="17" t="inlineStr">
-        <is>
-          <t>Audit row 20</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="C36" s="16">
+        <f>Audit!D27</f>
+        <v/>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>Audit row 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Findings that need a decision or a fix: see the 'Findings' sheet</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>The acceptance ties read from the system: see the 'Baselines' sheet</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="19" t="inlineStr">
-        <is>
-          <t>Source: The implementation agreement between MAIIC and Dupleix Institute, Schedule 1 (solution components; deliverables 5, 6 and 7 are the manuals). Spec v4 section 8 (the build plan) and section 12.</t>
+    <row r="40">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>Source: The implementation agreement between MAIIC and Dupleix Institute, Schedule 1 (solution components; deliverable 2 the migration reconciliation report; deliverables 5, 6 and 7 the manuals), as the manuals cite it. Spec v4 section 8 (the build plan, P4b to P10) and section 12.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A14:D14"/>
   </mergeCells>
-  <conditionalFormatting sqref="C14:C30">
+  <conditionalFormatting sqref="C14:C37">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$C14="Done"</formula>
     </cfRule>
@@ -1102,34 +1249,48 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B15" location="'Audit'!A6" display="Data onboarding"/>
+    <hyperlink ref="B15" location="'Audit'!A6" display="Data import and onboarding"/>
     <hyperlink ref="D15" location="'Audit'!A6" display="Audit row 6"/>
-    <hyperlink ref="B16" location="'Audit'!A7" display="Collateral management"/>
+    <hyperlink ref="B16" location="'Audit'!A7" display="Collateral module"/>
     <hyperlink ref="D16" location="'Audit'!A7" display="Audit row 7"/>
-    <hyperlink ref="B17" location="'Audit'!A8" display="The effective interest rate and revenue recognition"/>
+    <hyperlink ref="B17" location="'Audit'!A8" display="EIR module and revenue recognition"/>
     <hyperlink ref="D17" location="'Audit'!A8" display="Audit row 8"/>
-    <hyperlink ref="B18" location="'Audit'!A9" display="IFRS 9 model set-up"/>
+    <hyperlink ref="B18" location="'Audit'!A9" display="IFRS 9 model set-up: SICR and staging, PD, LGD, forward-looking information"/>
     <hyperlink ref="D18" location="'Audit'!A9" display="Audit row 9"/>
-    <hyperlink ref="B19" location="'Audit'!A10" display="The ECL engine"/>
+    <hyperlink ref="B19" location="'Audit'!A10" display="ECL engine"/>
     <hyperlink ref="D19" location="'Audit'!A10" display="Audit row 10"/>
     <hyperlink ref="B20" location="'Audit'!A11" display="Reports"/>
     <hyperlink ref="D20" location="'Audit'!A11" display="Audit row 11"/>
-    <hyperlink ref="B21" location="'Audit'!A12" display="The audit trail"/>
+    <hyperlink ref="B21" location="'Audit'!A12" display="Audit trail"/>
     <hyperlink ref="D21" location="'Audit'!A12" display="Audit row 12"/>
-    <hyperlink ref="B22" location="'Audit'!A13" display="The dashboard and the workspace"/>
+    <hyperlink ref="B22" location="'Audit'!A13" display="Dashboard and workspace"/>
     <hyperlink ref="D22" location="'Audit'!A13" display="Audit row 13"/>
-    <hyperlink ref="B23" location="'Audit'!A14" display="Administration"/>
+    <hyperlink ref="B23" location="'Audit'!A14" display="User and access management; operations"/>
     <hyperlink ref="D23" location="'Audit'!A14" display="Audit row 14"/>
-    <hyperlink ref="B25" location="'Audit'!A16" display="User manual"/>
+    <hyperlink ref="B24" location="'Audit'!A15" display="Internal grading"/>
+    <hyperlink ref="D24" location="'Audit'!A15" display="Audit row 15"/>
+    <hyperlink ref="B25" location="'Audit'!A16" display="EAD module"/>
     <hyperlink ref="D25" location="'Audit'!A16" display="Audit row 16"/>
-    <hyperlink ref="B26" location="'Audit'!A17" display="Administrator manual"/>
+    <hyperlink ref="B26" location="'Audit'!A17" display="Support"/>
     <hyperlink ref="D26" location="'Audit'!A17" display="Audit row 17"/>
-    <hyperlink ref="B27" location="'Audit'!A18" display="Technical manual and installation guide"/>
+    <hyperlink ref="B27" location="'Audit'!A18" display="The Mega Farm programme"/>
     <hyperlink ref="D27" location="'Audit'!A18" display="Audit row 18"/>
-    <hyperlink ref="B29" location="'Audit'!A20" display="The specification's acceptance tests"/>
-    <hyperlink ref="D29" location="'Audit'!A20" display="Audit row 20"/>
-    <hyperlink ref="A31" location="'Findings'!A1" display="Findings that need a decision or a fix: see the 'Findings' sheet"/>
-    <hyperlink ref="A32" location="'Baselines'!A1" display="The acceptance ties read from the system: see the 'Baselines' sheet"/>
+    <hyperlink ref="B28" location="'Audit'!A19" display="Annual report alignment"/>
+    <hyperlink ref="D28" location="'Audit'!A19" display="Audit row 19"/>
+    <hyperlink ref="B30" location="'Audit'!A21" display="Migration reconciliation report"/>
+    <hyperlink ref="D30" location="'Audit'!A21" display="Audit row 21"/>
+    <hyperlink ref="B31" location="'Audit'!A22" display="User manual"/>
+    <hyperlink ref="D31" location="'Audit'!A22" display="Audit row 22"/>
+    <hyperlink ref="B32" location="'Audit'!A23" display="Administrator and Technical Manual"/>
+    <hyperlink ref="D32" location="'Audit'!A23" display="Audit row 23"/>
+    <hyperlink ref="B33" location="'Audit'!A24" display="Installation and Configuration Guide"/>
+    <hyperlink ref="D33" location="'Audit'!A24" display="Audit row 24"/>
+    <hyperlink ref="B34" location="'Audit'!A25" display="Deployment, training and source code"/>
+    <hyperlink ref="D34" location="'Audit'!A25" display="Audit row 25"/>
+    <hyperlink ref="B36" location="'Audit'!A27" display="The specification's acceptance tests"/>
+    <hyperlink ref="D36" location="'Audit'!A27" display="Audit row 27"/>
+    <hyperlink ref="A38" location="'Findings'!A1" display="Findings that need a decision or a fix: see the 'Findings' sheet"/>
+    <hyperlink ref="A39" location="'Baselines'!A1" display="The acceptance ties read from the system: see the 'Baselines' sheet"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1143,7 +1304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1169,7 +1330,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>Malawi Agricultural and Industrial Investment Company (MAIIC) - IFRS 9 EIR and ECL system - build of 8 October 2026 against specification v4. Prepared 9 October 2026 from the build of specification v4 and the system as it stands on the clean install. The clause numbers of the signed schedule are to be confirmed at acceptance (P9). Reviewer: Dr Thomson Kumwenda (CFO), at acceptance. Status definitions: see 'Contents'.</t>
+          <t>Malawi Agricultural and Industrial Investment Company (MAIIC) - IFRS 9 EIR and ECL system - build of 14 October 2026 (branch eir_revenue_recognition, commit abe140d) against specification v4. As of 14 October 2026: the code at commit abe140d (branch eir_revenue_recognition) and the fresh bootstrap maiic_ifrs9_results2 of 13 October 2026 (made before commit 216aee2), read with SELECTs only. The clause numbers of the signed schedule are to be confirmed at acceptance (P9); the deliverable numbers are those the manuals carry. Reviewer: Dr Thomson Kumwenda (CFO), at acceptance. Status definitions: see 'Contents'.</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1413,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>Data onboarding</t>
+          <t>Data import and onboarding</t>
         </is>
       </c>
       <c r="C6" s="22" t="inlineStr">
@@ -1267,7 +1428,7 @@
       </c>
       <c r="E6" s="22" t="inlineStr">
         <is>
-          <t>The E-Banker landing zone with its gates, the loan book built from the ledger by three methods, the take-on schedules landed with their cells, the trial balances; the bootstrap loads it all from the committed folder and proves it against the golden numbers.</t>
+          <t>The E-Banker landing zone with its gates (hash, row count, query register, dates, keys); packs 2 to 4 land in the bootstrap (Bootstrap::landLaterPacks); the loan book built from the ledger for every month from July 2024; the take-on workbook landed cell by cell; the monthly trial balances through their own screen (EIR Data, Trial Balances; TrialBalanceLandingService); every import has a sample file and a check that refuses a bad file before anything is written. Feed routes 1 to 3 are built (manual upload, folder poll, API inbox); routes 4 and 5 are catalogue options only.</t>
         </is>
       </c>
       <c r="F6" s="22" t="inlineStr"/>
@@ -1278,7 +1439,7 @@
       </c>
       <c r="H6" s="22" t="inlineStr">
         <is>
-          <t>Data Foundation, E-Banker Feed: /eir-feed; Take-on Schedules: /eir-takeon</t>
+          <t>Customer &amp; Loan Data, Imports &amp; Feeds: /imports, /eir-feed, /eir-takeon; EIR Data, Trial Balances: /eir-trial-balances</t>
         </is>
       </c>
       <c r="I6" s="22" t="inlineStr"/>
@@ -1289,7 +1450,7 @@
       </c>
       <c r="K6" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Ebanker\PackLandingServiceTest; Tests\Feature\Ebanker\LoanBookBuildServiceTest</t>
+          <t>Tests\Feature\Ebanker\PackLandingServiceTest::test_a_tampered_hash_quarantines_the_pack_and_keeps_its_rows_where_no_reader_sees_them; Tests\Feature\Ebanker\TrialBalanceLandingServiceTest; Tests\Feature\Imports\ImportValidationTest::test_the_check_endpoint_writes_nothing_and_a_clean_file_passes</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1462,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>Collateral management</t>
+          <t>Collateral module</t>
         </is>
       </c>
       <c r="C7" s="22" t="inlineStr">
@@ -1316,25 +1477,29 @@
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>The collateral register, types and allocation screens exist; the security register from E-Banker (P2_11) is landed; 31 active accounts have no security recorded.</t>
-        </is>
-      </c>
-      <c r="F7" s="22" t="inlineStr"/>
+          <t>The collateral register, types and allocation screens exist with a checked import; the E-Banker security register (P2_11, 185 rows) is landed. On the fresh bootstrap collateral_registers and collateral_allocations are empty, and the LGD engine reads no collateral. An uncommitted migration (collateral type code as text) is in the working tree.</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Fresh bootstrap maiic_ifrs9_results2 (13 October 2026, before commit 216aee2).</t>
+        </is>
+      </c>
       <c r="G7" s="22" t="inlineStr">
         <is>
-          <t>Partially done: the data is Credit's to complete.</t>
+          <t>Partially done: Credit completes the data; Dupleix links collateral to the LGD.</t>
         </is>
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>Data Foundation, Collateral Register: /collateral/register</t>
+          <t>Collateral Management, Collateral Register: /collateral/register</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr"/>
       <c r="J7" s="22" t="inlineStr"/>
       <c r="K7" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Ebanker\PackLandingServiceTest::test_a_composite_key_lands_one_row_per_pair</t>
+          <t>Tests\Feature\Imports\ImportValidationTest::test_a_collateral_file_missing_a_required_column_is_refused_and_nothing_is_written</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1511,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>The effective interest rate and revenue recognition</t>
+          <t>EIR module and revenue recognition</t>
         </is>
       </c>
       <c r="C8" s="22" t="inlineStr">
@@ -1356,34 +1521,38 @@
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Partially done</t>
         </is>
       </c>
       <c r="E8" s="22" t="inlineStr">
         <is>
-          <t>The EIR engine, the roll-forward with cash from the ledger, the GL reconciliation, the EIR as at any date; 31 EIRs solved on the clean install, 12 locked, 19 awaiting the fee rulebook's approval.</t>
-        </is>
-      </c>
-      <c r="F8" s="22" t="inlineStr"/>
+          <t>Built: the EIR solver on dated flows (tranche-timed and take-on EIRs, 216aee2), the fee routes with source precedence, the monthly roll-forward with ledger cash, the GL reconciliation, the EIR as at any date, write-offs classified. Not built: modification and restructuring (5.4.3, 3.3.2), the B5.4.6 catch-up, rate reset events, the journal proposal (D6). On the fresh bootstrap 14 of 144 EIRs are locked, 33 are blocked at the fee gate and 97 have no approved schedule.</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>Fresh bootstrap maiic_ifrs9_results2 (13 October 2026, before commit 216aee2). Until 14 October 2026 this row was Done and said '31 solved, 12 locked, 19 awaiting'.</t>
+        </is>
+      </c>
       <c r="G8" s="22" t="inlineStr">
         <is>
-          <t>Compliant in mechanics; see the IFRS 9 EIR workbook's findings.</t>
+          <t>Partially done; see the IFRS 9 EIR workbook.</t>
         </is>
       </c>
       <c r="H8" s="22" t="inlineStr">
         <is>
-          <t>Financial Modelling, EIR Calculations: /eir-calculations; Report Hub, EIR as at a Date: /eir-as-at</t>
+          <t>EIR &amp; Revenue Recognition: /eir-calculations; /eir-as-at; /eir-reconciliation</t>
         </is>
       </c>
       <c r="I8" s="22" t="inlineStr"/>
       <c r="J8" s="22" t="inlineStr">
         <is>
-          <t>(section 4.2)</t>
+          <t>day_count; stage3_interest_basis; fee_source_precedence; takeon_eir_plausibility; partly_drawn_interest_basis</t>
         </is>
       </c>
       <c r="K8" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Eir\EirCalculationWorkflowTest; Tests\Feature\Eir\EirAsAtServiceTest</t>
+          <t>Tests\Feature\Eir\EirCalculationWorkflowTest; Tests\Feature\Eir\EirAsAtServiceTest; Tests\Feature\Eir\TakeonAndTrancheEirInputTest</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1564,7 @@
       </c>
       <c r="B9" s="22" t="inlineStr">
         <is>
-          <t>IFRS 9 model set-up</t>
+          <t>IFRS 9 model set-up: SICR and staging, PD, LGD, forward-looking information</t>
         </is>
       </c>
       <c r="C9" s="22" t="inlineStr">
@@ -1410,10 +1579,14 @@
       </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>The staging thresholds per the directive, the PD transition matrix and the LGD cohort workout as services, the forward-looking chain (correlation, regression, guardrail), the transmission methods with their cards, the scenario sets, all governed in the Governance Centre with 48 settings.</t>
-        </is>
-      </c>
-      <c r="F9" s="22" t="inlineStr"/>
+          <t>Staging on the directive's thresholds (seeded rows, read-only on screen) with the governed day basis, missed-instalment trigger and cure period, reading E-Banker's instalment chart in force (216aee2); PD and LGD by segment on the governed basis, Mega Farm kept apart; the forward-looking chain (correlation, regression, guardrail), the transmission methods with their cards, the scenario sets; all governed in the Governance Centre, whose catalogue holds 61 settings (20 of which no engine reads; IFRS 9 EIR workbook S4).</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>Until 14 October 2026 the row said 48 settings.</t>
+        </is>
+      </c>
       <c r="G9" s="22" t="inlineStr">
         <is>
           <t>Compliant.</t>
@@ -1421,18 +1594,18 @@
       </c>
       <c r="H9" s="22" t="inlineStr">
         <is>
-          <t>Governance Centre: /eir-governance; Financial Modelling: /expected-credit-loss</t>
+          <t>IFRS 9 Model Setup; Forward-Looking Information; Governance Centre: /eir-governance</t>
         </is>
       </c>
       <c r="I9" s="22" t="inlineStr"/>
       <c r="J9" s="22" t="inlineStr">
         <is>
-          <t>(section 4.2)</t>
+          <t>dpd_basis; stage3_missed_instalments; stage_cure_months; pd_segmentation_basis; lgd_segment_min_cohort; fli_transmission_method</t>
         </is>
       </c>
       <c r="K9" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Eir\GovernanceServiceTest; Tests\Feature\Pd\PdAndLgdEngineTest; Tests\Feature\FLI\FliRouteServiceTest</t>
+          <t>Tests\Feature\Eir\GovernanceServiceTest; Tests\Feature\Pd\PdAndLgdEngineTest; Tests\Feature\Pd\PdSegmentationTest; Tests\Feature\FLI\FliRouteServiceTest</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1617,7 @@
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>The ECL engine</t>
+          <t>ECL engine</t>
         </is>
       </c>
       <c r="C10" s="22" t="inlineStr">
@@ -1454,23 +1627,27 @@
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Partially done</t>
         </is>
       </c>
       <c r="E10" s="22" t="inlineStr">
         <is>
-          <t>The time-phased ECL discounted at the EIR, on the post-FLI PD, with the sensitivity across scenarios and the stress runs; on the clean install 8.94bn at August 2026 under the bootstrap label.</t>
-        </is>
-      </c>
-      <c r="F10" s="22" t="inlineStr"/>
+          <t>The ECL per loan on the post-FLI PD, weighted across the scenarios, for every period, failing closed on a missing input; since 216aee2 the month-end runs discounted at the EIR and stores the discounted allowance beside the undiscounted measure. The reports and the IFRS 9 note still read the undiscounted ecl_value. On the fresh bootstrap the main book at September 2026 carries 11.57bn undiscounted and 7.12bn discounted on the 62 loans resolved (72 unresolved, before 216aee2).</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>Fresh bootstrap maiic_ifrs9_results2 (13 October 2026, before commit 216aee2). Until 14 October 2026 this row was Done and quoted 8.94bn.</t>
+        </is>
+      </c>
       <c r="G10" s="22" t="inlineStr">
         <is>
-          <t>Compliant; the figures await MAIIC's reviews (fee rulebook, matrix and LGD key-locks, the fit and the set).</t>
+          <t>Partially done: the reports must carry the discounted allowance; the figures await MAIIC's reviews.</t>
         </is>
       </c>
       <c r="H10" s="22" t="inlineStr">
         <is>
-          <t>Financial Modelling, ECL Calculation: /expected-credit-loss</t>
+          <t>ECL Processing, ECL Calculation: /expected-credit-loss/list</t>
         </is>
       </c>
       <c r="I10" s="22" t="inlineStr"/>
@@ -1481,7 +1658,7 @@
       </c>
       <c r="K10" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Ecl\TimePhasedEclServiceTest; Tests\Feature\Scenario\ScenarioSetServiceTest</t>
+          <t>Tests\Feature\Ecl\TimePhasedEclServiceTest; Tests\Feature\Ecl\EclGoldenNumberTest::discounted_mode_keeps_undiscounted_ecl_and_names_unresolved_contracts; Tests\Feature\Scenario\ScenarioSetServiceTest</t>
         </is>
       </c>
     </row>
@@ -1508,25 +1685,29 @@
       </c>
       <c r="E11" s="22" t="inlineStr">
         <is>
-          <t>Thirty reports in the Report Hub, every one rendered by ifrs9:smoke-reports on the clean install; the EIR as at a date with its CSV; the auditor's pack.</t>
-        </is>
-      </c>
-      <c r="F11" s="22" t="inlineStr"/>
+          <t>29 reports in the Reports hub, each rendered by ifrs9:smoke-reports and downloadable as PDF and Excel; the IFRS 9 note; the RBM Return (provisional); the EIR as at a date and the GL reconciliation with their exports; the loan book and ECL reconciliations; stress testing; the auditor's pack. Content gaps are audited in the IFRS 7 and RBM workbooks (write-offs nil, undiscounted allowance, provisional return form).</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>Until 14 October 2026 the row said thirty reports and cited an unrelated test.</t>
+        </is>
+      </c>
       <c r="G11" s="22" t="inlineStr">
         <is>
-          <t>Compliant.</t>
+          <t>Compliant as a component.</t>
         </is>
       </c>
       <c r="H11" s="22" t="inlineStr">
         <is>
-          <t>Report Hub: /ifrs9-reports</t>
+          <t>Reports: /ifrs9-reports; /rbm-return; /auditor-pack</t>
         </is>
       </c>
       <c r="I11" s="22" t="inlineStr"/>
       <c r="J11" s="22" t="inlineStr"/>
       <c r="K11" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Eir\EirAsAtServiceTest</t>
+          <t>Tests\Feature\Ifrs9ReportDownloadTest::test_report_downloads_as_pdf; Tests\Feature\Pd\SegmentReportsRenderTest::test_the_reports_with_the_pd_parts_render_and_download</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1719,7 @@
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>The audit trail</t>
+          <t>Audit trail</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
@@ -1553,7 +1734,7 @@
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>The audit log records every load, build, approval, staging, engine run, setting change and compliance sign-off with the old and new values; the Governance Centre's maker-checker is enforced in code.</t>
+          <t>The audit log records every load, build, approval, staging, engine run, setting change, write-off and compliance sign-off with the old and new values; the Audit Trace follows one record; the Governance Centre's maker-checker is enforced in code.</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr"/>
@@ -1564,14 +1745,18 @@
       </c>
       <c r="H12" s="22" t="inlineStr">
         <is>
-          <t>Governance Centre, Audit Trail: /audit-trail</t>
+          <t>Governance, Audit: Audit Trail /audit-trail; Audit Trace /audit-trace; Compliance Audits /compliance-audits</t>
         </is>
       </c>
       <c r="I12" s="22" t="inlineStr"/>
-      <c r="J12" s="22" t="inlineStr"/>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>maker_checker_admin_override</t>
+        </is>
+      </c>
       <c r="K12" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\Eir\EirGovernanceControllerTest</t>
+          <t>Tests\Feature\Eir\GovernanceServiceTest::test_every_proposal_and_approval_is_audit_logged_with_old_and_new_values; Tests\Feature\Compliance\ComplianceAuditServiceTest</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1768,7 @@
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>The dashboard and the workspace</t>
+          <t>Dashboard and workspace</t>
         </is>
       </c>
       <c r="C13" s="22" t="inlineStr">
@@ -1598,7 +1783,7 @@
       </c>
       <c r="E13" s="22" t="inlineStr">
         <is>
-          <t>The dashboard and the workspace exist under the suite layout with light and dark mode.</t>
+          <t>The dashboard (period, portfolio and compare-to filters; ECL by portfolio, scenarios by stage and observed default-rate charts, each with its own range) and the workspace of the period's tasks, in light and dark mode.</t>
         </is>
       </c>
       <c r="F13" s="22" t="inlineStr"/>
@@ -1616,7 +1801,7 @@
       <c r="J13" s="22" t="inlineStr"/>
       <c r="K13" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\NavigationTest</t>
+          <t>Tests\Feature\DashboardChartsTest::test_every_month_of_ecl_by_portfolio_adds_back_to_the_trend_total</t>
         </is>
       </c>
     </row>
@@ -1628,12 +1813,12 @@
       </c>
       <c r="B14" s="22" t="inlineStr">
         <is>
-          <t>Administration</t>
+          <t>User and access management; operations</t>
         </is>
       </c>
       <c r="C14" s="22" t="inlineStr">
         <is>
-          <t>Users, roles and permissions, settings, support.</t>
+          <t>Users, roles and permissions, settings, financial periods, maintenance.</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
@@ -1643,10 +1828,14 @@
       </c>
       <c r="E14" s="22" t="inlineStr">
         <is>
-          <t>User management, roles and permissions, settings and support tickets; the navigation is filtered by permission so no user sees a link that answers 403.</t>
-        </is>
-      </c>
-      <c r="F14" s="22" t="inlineStr"/>
+          <t>User management, roles and permissions, settings, financial periods and the Maintenance screen that runs the month-end jobs; every route requires a login and the navigation is filtered by permission so no user sees a link that answers 403.</t>
+        </is>
+      </c>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>Until 14 October 2026 the path given was /users; the route is /user.</t>
+        </is>
+      </c>
       <c r="G14" s="22" t="inlineStr">
         <is>
           <t>Compliant.</t>
@@ -1654,220 +1843,567 @@
       </c>
       <c r="H14" s="22" t="inlineStr">
         <is>
-          <t>Administration: /users</t>
+          <t>Access &amp; Setup, Users &amp; Roles: /user, /user/role; Settings: /setting; Support &amp; Maintenance, Maintenance: /maintenance</t>
         </is>
       </c>
       <c r="I14" s="22" t="inlineStr"/>
       <c r="J14" s="22" t="inlineStr"/>
       <c r="K14" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\NavigationTest::test_every_leaf_names_a_registered_route</t>
+          <t>Tests\Feature\NavigationTest::test_every_leaf_names_a_registered_route; Tests\Feature\Security\RequireLoginTest::test_no_get_route_answers_a_guest_with_a_page</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>DOCUMENTATION</t>
-        </is>
-      </c>
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>S1.10</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Internal grading</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Internal credit grades for the book, linked to the PD.</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Partially done</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
+        <is>
+          <t>The Internal Grades screens (profiles, the PD matrix with each grade's S&amp;P rating) and the S&amp;P grades import exist (SpGradesImportService). No engine reads the grades: on the fresh bootstrap there are 0 internal grade profiles and internal_grade_code is null on every main-book loan; staging and PD run on days past due and segments.</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Fresh bootstrap maiic_ifrs9_results2 (13 October 2026, before commit 216aee2). Row added 14 October 2026.</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>Partially done: MAIIC decides whether grades drive the PD; until then they are reference only.</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>IFRS 9 Model Setup, PD Model, Internal Grades: /internal-grading</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="inlineStr"/>
+      <c r="J15" s="22" t="inlineStr"/>
+      <c r="K15" s="22" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="22" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>S1.11</t>
         </is>
       </c>
       <c r="B16" s="22" t="inlineStr">
         <is>
-          <t>User manual</t>
+          <t>EAD module</t>
         </is>
       </c>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>A user manual for the finance officer.</t>
+          <t>Exposure at default per facility.</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Partially done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>The help centre carries the user manual with per-page help and a PDF; the navigation chapter and screenshots are to be redone for the suite layout.</t>
-        </is>
-      </c>
-      <c r="F16" s="22" t="inlineStr"/>
+          <t>EAD is the carrying amount plus undrawn commitments times utilisation, floored at nil; an undrawn amount past maturity is no exposure (216aee2); the EAD report renders.</t>
+        </is>
+      </c>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>Row added 14 October 2026.</t>
+        </is>
+      </c>
       <c r="G16" s="22" t="inlineStr">
         <is>
-          <t>Partially done.</t>
+          <t>Compliant.</t>
         </is>
       </c>
       <c r="H16" s="22" t="inlineStr">
         <is>
-          <t>System Documentation, User Manual: /help</t>
+          <t>Reports: EAD /ifrs9-reports/ead-report</t>
         </is>
       </c>
       <c r="I16" s="22" t="inlineStr"/>
       <c r="J16" s="22" t="inlineStr"/>
       <c r="K16" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\NavigationTest</t>
+          <t>Tests\Feature\Ebanker\LoanBookBuildServiceTest::test_an_undrawn_amount_past_maturity_is_no_exposure; Tests\Feature\Ecl\EclBuildUpServiceTest::test_a_credit_balance_has_no_exposure_and_no_negative_ecl</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="22" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>S1.12</t>
         </is>
       </c>
       <c r="B17" s="22" t="inlineStr">
         <is>
-          <t>Administrator manual</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="C17" s="22" t="inlineStr">
         <is>
-          <t>An administrator manual.</t>
+          <t>Support tickets with a trail.</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Partially done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E17" s="22" t="inlineStr">
         <is>
-          <t>The administrator manual exists in the help centre; the passages naming the old menu groups are to be re-worded.</t>
-        </is>
-      </c>
-      <c r="F17" s="22" t="inlineStr"/>
+          <t>Support tickets with references, status changes recorded in the activity trail and resolution dates.</t>
+        </is>
+      </c>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>Row added 14 October 2026.</t>
+        </is>
+      </c>
       <c r="G17" s="22" t="inlineStr">
         <is>
-          <t>Partially done.</t>
+          <t>Compliant.</t>
         </is>
       </c>
       <c r="H17" s="22" t="inlineStr">
         <is>
-          <t>System Documentation, Administrator Manual: /help/admin</t>
+          <t>Support &amp; Maintenance, Support Tickets: /tickets</t>
         </is>
       </c>
       <c r="I17" s="22" t="inlineStr"/>
       <c r="J17" s="22" t="inlineStr"/>
       <c r="K17" s="22" t="inlineStr">
         <is>
-          <t>Tests\Feature\NavigationTest</t>
+          <t>Tests\Feature\TicketsTest::test_status_change_is_recorded_in_the_activity_trail</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
+          <t>S1.13</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>The Mega Farm programme</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>The Government's Mega Farm loans provided for on a documented basis, separately from MAIIC's own book.</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Evidence needed from MAIIC</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
+        <is>
+          <t>Since 216aee2 the programme is segmented as its own portfolio, kept out of MAIIC's PD, LGD and ECL, and provided by megafarm:ecl from its own LGD cohort under the governed PD method; its monthly books (MF_01, MF_03) are landed. Not built: the interest split, the maize receivable and the fund liability of spec 16.4 and 16.5, which wait on D30.</t>
+        </is>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>Row added 14 October 2026. The IFRS 9 impairment workbook row 16 carries the detail.</t>
+        </is>
+      </c>
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>Evidence needed: Dr Thom's confirmation of D30.</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>ECL Processing, Mega Farm Programme: /megafarm</t>
+        </is>
+      </c>
+      <c r="I18" s="22" t="inlineStr"/>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>mega_farms_scope; megafarm_pd_method; megafarm_scalar_ceiling</t>
+        </is>
+      </c>
+      <c r="K18" s="22" t="inlineStr">
+        <is>
+          <t>Tests\Feature\Ecl\MegaFarmProgrammeSeparationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>S1.14</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Annual report alignment</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Stage tables by segment matching Note 8 of the audited statements (Mega Farm and the main book: gross, ECL and net by stage with the roll-forward), the sector concentration, interest income lines matching Note 15 and the RBM prudential tables (technical manual 7.6).</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Partially done</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>The IFRS 9 note gives gross, ECL and net by stage with the roll-forward for a chosen portfolio and ties every column; the concentration report; the RBM Return. Gaps: write-offs nil in the roll-forward, the allowance undiscounted, EIR interest only on locked loans, the RBM Return provisional.</t>
+        </is>
+      </c>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>Row added 14 October 2026.</t>
+        </is>
+      </c>
+      <c r="G19" s="22" t="inlineStr">
+        <is>
+          <t>Partially done; see the IFRS 7 and RBM workbooks.</t>
+        </is>
+      </c>
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>Reports: IFRS 9 note /ifrs9-reports/fs-disclosure; /rbm-return</t>
+        </is>
+      </c>
+      <c r="I19" s="22" t="inlineStr"/>
+      <c r="J19" s="22" t="inlineStr"/>
+      <c r="K19" s="22" t="inlineStr">
+        <is>
+          <t>Tests\Unit\EclMovementAttributionTest::test_every_column_ties</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>DELIVERABLES</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Migration reconciliation report</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>A reconciliation of the migrated data to the source system and the ledger.</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Partially done</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>The evidence exists in the system: the derived carrying amount equals E-Banker's own report on 2,495 of 2,495 in-scope account-months, the loan GLs tie to the December 2025 trial balance (two accepted exceptions), the interest posted ties to the ledger (Baselines sheet), and the Imports exception files, the Coverage and Blockers export and the trial balance output (installation guide 9.7). It is not assembled as one report, and the take-on fee totals stated by MAIIC and landed are not reconciled in it.</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>Fresh bootstrap maiic_ifrs9_results2 (13 October 2026, before commit 216aee2). Row added 14 October 2026.</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Partially done: assemble and sign the report.</t>
+        </is>
+      </c>
+      <c r="H21" s="22" t="inlineStr">
+        <is>
+          <t>Baselines sheet; EIR Calculations, Blockers: /eir-coverage; Imports: /imports</t>
+        </is>
+      </c>
+      <c r="I21" s="22" t="inlineStr"/>
+      <c r="J21" s="22" t="inlineStr"/>
+      <c r="K21" s="22" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>User manual</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>A user manual for the finance officer.</t>
+        </is>
+      </c>
+      <c r="D22" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>The help centre carries the user manual with per-page help and a PDF, including the Trial Balances and Write-offs screens of 13 October 2026; its chapter titles follow the suite groups.</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>Screenshots of the screens changed on 13 and 14 October were not checked for this audit. Until 14 October 2026 this row was Partially done.</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Compliant.</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Support &amp; Maintenance, System Documentation, User Manual: /help</t>
+        </is>
+      </c>
+      <c r="I22" s="22" t="inlineStr"/>
+      <c r="J22" s="22" t="inlineStr"/>
+      <c r="K22" s="22" t="inlineStr">
+        <is>
+          <t>Tests\Feature\HelpManualTest::test_pdf_renders_from_the_same_rows; Tests\Feature\AuditFindingM16ScreensTest::test_the_help_chapters_carry_the_suite_group_names</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Administrator and Technical Manual</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>The administrator manual and the technical manual (deliverable 6 in two volumes).</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Partially done</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>The administrator volume is in the help centre with its own PDF; the technical volume is repository Markdown under docs/manuals/technical rendered at /system-docs/technical. The technical volume does not yet describe the services of 13 and 14 October (WriteOffClassifier and the write-off register, TrialBalanceLandingService, Bootstrap::landLaterPacks, InstalmentChartHistory, the GL fee route and fee_source_precedence).</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>Until 14 October 2026 this workbook called D6 the administrator manual alone and D7 the technical manual with the installation guide, against DocumentFrontMatter.</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Partially done: the technical volume needs the new services.</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>System Documentation: Administrator Manual /help/admin; Technical Manual /system-docs/technical</t>
+        </is>
+      </c>
+      <c r="I23" s="22" t="inlineStr"/>
+      <c r="J23" s="22" t="inlineStr"/>
+      <c r="K23" s="22" t="inlineStr">
+        <is>
+          <t>Tests\Feature\HelpManualTest::test_admin_manual_reader_shows_only_admin_chapters_and_exports_pdf; Tests\Feature\SystemDocsTest::test_technical_manual_renders_chapters_with_anchored_sections_and_live_schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
-        <is>
-          <t>Technical manual and installation guide</t>
-        </is>
-      </c>
-      <c r="C18" s="22" t="inlineStr">
-        <is>
-          <t>A technical manual and an installation guide.</t>
-        </is>
-      </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Installation and Configuration Guide</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>An installation and configuration guide.</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
-        <is>
-          <t>Both are repository Markdown under docs/manuals, rendered in the system; the installation guide's section 9.8 gives the bootstrap and the monthly feed as the procedure.</t>
-        </is>
-      </c>
-      <c r="F18" s="22" t="inlineStr"/>
-      <c r="G18" s="22" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>Repository Markdown under docs/manuals/installation, rendered at /system-docs/installation with a PDF; section 9.8 gives the bootstrap and the monthly close as the procedure.</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>Section 9.8 step 3 does not yet name the later packs the bootstrap lands (packs 3 and 4). Until 14 October 2026 the paths given were /docs/technical and /docs/installation.</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
         <is>
           <t>Compliant.</t>
         </is>
       </c>
-      <c r="H18" s="22" t="inlineStr">
-        <is>
-          <t>System Documentation, Technical Manual: /docs/technical; Installation Guide: /docs/installation</t>
-        </is>
-      </c>
-      <c r="I18" s="22" t="inlineStr"/>
-      <c r="J18" s="22" t="inlineStr"/>
-      <c r="K18" s="22" t="inlineStr">
-        <is>
-          <t>Tests\Feature\NavigationTest</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>System Documentation, Installation Guide: /system-docs/installation</t>
+        </is>
+      </c>
+      <c r="I24" s="22" t="inlineStr"/>
+      <c r="J24" s="22" t="inlineStr"/>
+      <c r="K24" s="22" t="inlineStr">
+        <is>
+          <t>Tests\Feature\SystemDocsTest::test_installation_guide_renders_without_schema_appendix; Tests\Feature\SystemDocsTest::test_documentation_menu_lists_all_four_deliverables</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Deployment, training and source code</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>Install in MAIIC's environment; train MAIIC's users; hand over the source code (spec v4 section 8, P10).</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>Outstanding</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>Not started: the system runs on Dupleix's environment; no MAIIC user training has been delivered (docs/training holds a developer course, uncommitted); the read-only E-Banker account from ICT is awaited.</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>Row added 14 October 2026.</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>Outstanding (Dupleix, after P9).</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr"/>
+      <c r="I25" s="22" t="inlineStr"/>
+      <c r="J25" s="22" t="inlineStr"/>
+      <c r="K25" s="22" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>ACCEPTANCE</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B20" s="22" t="inlineStr">
+      <c r="B27" s="22" t="inlineStr">
         <is>
           <t>The specification's acceptance tests</t>
         </is>
       </c>
-      <c r="C20" s="22" t="inlineStr">
+      <c r="C27" s="22" t="inlineStr">
         <is>
           <t>The baselines of specification section 9 pass on the production copy.</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D27" s="23" t="inlineStr">
         <is>
           <t>Partially done</t>
         </is>
       </c>
-      <c r="E20" s="22" t="inlineStr">
-        <is>
-          <t>Nine golden checks pass on the clean install (the Baselines sheet of every workbook); the ECL at the year-ends and the revenue shift become golden numbers on the first run Dr Thom approves.</t>
-        </is>
-      </c>
-      <c r="F20" s="22" t="inlineStr"/>
-      <c r="G20" s="22" t="inlineStr">
-        <is>
-          <t>Partially done: the year-end golden numbers await MAIIC's decisions.</t>
-        </is>
-      </c>
-      <c r="H20" s="22" t="inlineStr">
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>eir:baselines and eir:bootstrap --verify assert: the interest posted January 2025 to July 2026, the method B tie on every in-scope account-month, the two year-end batch contras and the December 2025 loan GLs against the trial balance; all pass on the fresh bootstrap (Baselines sheet). Spec section 9 lists 16 ties; the rest, and the ECL and revenue-shift golden numbers, are not asserted.</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>Until 14 October 2026 the row said nine golden checks.</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>Partially done: the remaining ties and the golden numbers await MAIIC's first approved run.</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
         <is>
           <t>eir:bootstrap --verify; eir:baselines</t>
         </is>
       </c>
-      <c r="I20" s="22" t="inlineStr"/>
-      <c r="J20" s="22" t="inlineStr"/>
-      <c r="K20" s="22" t="inlineStr">
-        <is>
-          <t>Tests\Feature\Ebanker\LoanBookBuildServiceTest</t>
+      <c r="I27" s="22" t="inlineStr"/>
+      <c r="J27" s="22" t="inlineStr"/>
+      <c r="K27" s="22" t="inlineStr">
+        <is>
+          <t>Tests\Feature\Ebanker\LoanBookBuildServiceTest::test_method_b_derives_the_carrying_amount_from_the_ledger_and_keeps_the_stored_figure_beside_it</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K20"/>
+  <autoFilter ref="A4:K27"/>
   <mergeCells count="4">
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A26:K26"/>
     <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A20:K20"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:D20">
+  <conditionalFormatting sqref="D5:D27">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$D5="Done"</formula>
     </cfRule>
@@ -1884,13 +2420,13 @@
       <formula>$D5="Evidence needed from MAIIC"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K20">
+  <conditionalFormatting sqref="K5:K27">
     <cfRule type="expression" priority="6" dxfId="2">
       <formula>AND($D5="Done",$K5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Done,Partially done,Outstanding,Not applicable, documented,Evidence needed from MAIIC"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1909,7 +2445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1984,9 +2520,9 @@
           <t>F1</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>S1.1 to A1</t>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>S1.1</t>
         </is>
       </c>
       <c r="C5" s="22" t="inlineStr">
@@ -1996,7 +2532,7 @@
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>The rows follow the solution components the navigation was built on; the signed Schedule 1's numbering is not in the repository.</t>
+          <t>The rows follow the component list and deliverable numbers the manuals give for Schedule 1; the signed schedule is not in the repository.</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
@@ -2028,27 +2564,27 @@
       </c>
       <c r="B6" s="24" t="inlineStr">
         <is>
-          <t>D5, D6</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="C6" s="22" t="inlineStr">
         <is>
-          <t>The manuals name the old menu groups</t>
+          <t>The technical manual lags the build</t>
         </is>
       </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>Fifteen help-centre passages and the user manual's navigation chapter still refer to the groups the suite layout replaced.</t>
+          <t>The user manual's chapters carry the suite group names (the earlier finding on old menu groups is closed), but the technical volume does not describe the services of 13 and 14 October, and the installation guide's 9.8 does not name the later packs.</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr">
         <is>
-          <t>A reader is sent to a group that no longer exists.</t>
+          <t>A maintainer reading the manual misses the write-off, trial balance, chart-in-force and GL fee code.</t>
         </is>
       </c>
       <c r="F6" s="22" t="inlineStr">
         <is>
-          <t>Re-word the passages and retake the screenshots (spec 11.6).</t>
+          <t>Add the services to chapters 03, 04, 06 and 09 of the technical manual and the packs to installation 9.8.</t>
         </is>
       </c>
       <c r="G6" s="22" t="inlineStr">
@@ -2057,6 +2593,90 @@
         </is>
       </c>
       <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>The migration reconciliation report is not assembled</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>The ties exist (Baselines sheet, Coverage and Blockers, Imports exceptions, trial balance output) but no single signed report.</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Deliverable 2 cannot be accepted as one document.</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Assemble the report from the existing exports with the take-on fee reconciliation and present it for sign-off.</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Dupleix / Finance</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>Deployment and training not started</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>The system is not installed at MAIIC; no user training has been delivered.</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>Go-live on 31 October 2026 depends on it.</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>Agree the installation date and training plan with MAIIC ICT and Finance.</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Dupleix / MAIIC ICT</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -2064,13 +2684,16 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In progress,Closed,Deferred"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="A2" location="'Contents'!A1" display="Back to Contents"/>
-    <hyperlink ref="B6" location="'Audit'!A16" display="D5, D6"/>
+    <hyperlink ref="B5" location="'Audit'!A6" display="S1.1"/>
+    <hyperlink ref="B6" location="'Audit'!A23" display="D6"/>
+    <hyperlink ref="B7" location="'Audit'!A21" display="D2"/>
+    <hyperlink ref="B8" location="'Audit'!A25" display="P10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2084,7 +2707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="64" customWidth="1" min="1" max="1"/>
@@ -2112,7 +2735,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-09 00:03:09 from maiic_ifrs9_bootstrap. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
+          <t>Generated 2026-10-14 08:30:21 from maiic_ifrs9_results2. The PASS/FAIL in column E is a formula on columns B and C, so it recomputes if a figure is typed over.</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2795,7 @@
     <row r="6">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>Derived carrying amount against the stored report (over 2 cents)</t>
+          <t>Derived carrying amount against the stored report, in-scope loan GLs (over 2 cents)</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
@@ -2182,7 +2805,7 @@
       </c>
       <c r="C6" s="22" t="inlineStr">
         <is>
-          <t>0 of 2361 account-months</t>
+          <t>0 of 2495 account-months</t>
         </is>
       </c>
       <c r="D6" s="22" t="n">
@@ -2197,20 +2820,24 @@
     <row r="7">
       <c r="A7" s="22" t="inlineStr">
         <is>
-          <t>Year-end interest batch contra on 4215</t>
-        </is>
-      </c>
-      <c r="B7" s="25" t="n">
-        <v>32956675.55</v>
-      </c>
-      <c r="C7" s="25" t="n">
-        <v>32956675.55</v>
+          <t>Mega Farm: account-months whose MF_03 ledger differs from the Loan Book Report (reported, not a test)</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>reported</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>77540 account-months</t>
+        </is>
       </c>
       <c r="D7" s="22" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="E7" s="26">
-        <f>IF(ABS(B7-C7)&lt;=D7,"PASS","FAIL")</f>
+        <f>IF(B7=C7,"PASS","FAIL")</f>
         <v/>
       </c>
       <c r="F7" s="22" t="inlineStr"/>
@@ -2218,17 +2845,17 @@
     <row r="8">
       <c r="A8" s="22" t="inlineStr">
         <is>
-          <t>Year-end interest batch contra on 4216</t>
+          <t>Year-end interest batch contra on 4215</t>
         </is>
       </c>
       <c r="B8" s="25" t="n">
-        <v>-21733262.7</v>
+        <v>32956675.55</v>
       </c>
       <c r="C8" s="25" t="n">
-        <v>-21733262.7</v>
+        <v>32956675.55</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>0.01</v>
+        <v>1</v>
       </c>
       <c r="E8" s="26">
         <f>IF(ABS(B8-C8)&lt;=D8,"PASS","FAIL")</f>
@@ -2239,17 +2866,17 @@
     <row r="9">
       <c r="A9" s="22" t="inlineStr">
         <is>
-          <t>Loan book 1050101 at 31 Dec 2025 against the trial balance</t>
+          <t>Year-end interest batch contra on 4216</t>
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>1368737810.68</v>
+        <v>-21733262.7</v>
       </c>
       <c r="C9" s="25" t="n">
-        <v>1368737810.68</v>
+        <v>-21733262.7</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="E9" s="26">
         <f>IF(ABS(B9-C9)&lt;=D9,"PASS","FAIL")</f>
@@ -2260,14 +2887,14 @@
     <row r="10">
       <c r="A10" s="22" t="inlineStr">
         <is>
-          <t>Loan book 1050102 at 31 Dec 2025 against the trial balance</t>
+          <t>Loan book 1050101 at 31 Dec 2025 against the trial balance</t>
         </is>
       </c>
       <c r="B10" s="25" t="n">
-        <v>6434045052.56</v>
+        <v>1368737810.68</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>6434045052.56</v>
+        <v>1368737810.68</v>
       </c>
       <c r="D10" s="22" t="n">
         <v>1</v>
@@ -2281,14 +2908,14 @@
     <row r="11">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>Loan book 1050201 at 31 Dec 2025 against the trial balance (accepted exception, spec 3.5: -400,000.00)</t>
+          <t>Loan book 1050102 at 31 Dec 2025 against the trial balance</t>
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>1402393139.46</v>
+        <v>6434045052.56</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>1401993139.46</v>
+        <v>6434045052.56</v>
       </c>
       <c r="D11" s="22" t="n">
         <v>1</v>
@@ -2302,14 +2929,14 @@
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
         <is>
-          <t>Loan book 1050202 at 31 Dec 2025 against the trial balance (accepted exception, spec 3.5: 1,000,000.00)</t>
+          <t>Loan book 1050201 at 31 Dec 2025 against the trial balance (accepted exception, spec 3.5: -400,000.00)</t>
         </is>
       </c>
       <c r="B12" s="25" t="n">
-        <v>3808288656.15</v>
+        <v>1402393139.46</v>
       </c>
       <c r="C12" s="25" t="n">
-        <v>3809288656.15</v>
+        <v>1401993139.46</v>
       </c>
       <c r="D12" s="22" t="n">
         <v>1</v>
@@ -2323,14 +2950,14 @@
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t>Loan book 1050401 at 31 Dec 2025 against the trial balance</t>
+          <t>Loan book 1050202 at 31 Dec 2025 against the trial balance (accepted exception, spec 3.5: 1,000,000.00)</t>
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>1827148120.69</v>
+        <v>3808288656.15</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>1827148120.69</v>
+        <v>3809288656.15</v>
       </c>
       <c r="D13" s="22" t="n">
         <v>1</v>
@@ -2341,8 +2968,29 @@
       </c>
       <c r="F13" s="22" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>Loan book 1050401 at 31 Dec 2025 against the trial balance</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="n">
+        <v>1827148120.69</v>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>1827148120.69</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="26">
+        <f>IF(ABS(B14-C14)&lt;=D14,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="F14" s="22" t="inlineStr"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="E5:E13">
+  <conditionalFormatting sqref="E5:E14">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E5="PASS"</formula>
     </cfRule>

</xml_diff>